<commit_message>
Improve Stage 2 capstone guidance and materials
</commit_message>
<xml_diff>
--- a/CAPSTONE/bus311-capstone-revenue-analysis.xlsx
+++ b/CAPSTONE/bus311-capstone-revenue-analysis.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="Rb7da3582ef2d40af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revenue Map" sheetId="2" r:id="R3e735bf6fdca4a32"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revenue History" sheetId="3" r:id="R1c1c989598cb4284"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Driver Analysis" sheetId="4" r:id="R6507c0a5ca8649e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Peers &amp; Demand" sheetId="5" r:id="Rca40fd9c69da468b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Indicators &amp; Risks" sheetId="6" r:id="R3758d0bf074b4533"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hypothesis &amp; Scenarios" sheetId="7" r:id="Raef48f092689488e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="8" r:id="R4fe0d672e6394843"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks &amp; Submission" sheetId="9" r:id="Rc1aceb5a649e4c5b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="R7c51ae69d9974287"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revenue Map" sheetId="2" r:id="R708dacbc38ed4060"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revenue History" sheetId="3" r:id="R2c9775b80ad64d97"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Driver Analysis" sheetId="4" r:id="Rea58d6440647434a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Peers &amp; Demand" sheetId="5" r:id="Rc045058e62404d45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Indicators &amp; Risks" sheetId="6" r:id="Rfc3be910c1ec484f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hypothesis &amp; Scenarios" sheetId="7" r:id="R889a4b282d8d491e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="8" r:id="R8c379b24f85a4e7b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks &amp; Submission" sheetId="9" r:id="Ra821774f4a5c429d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -838,7 +838,7 @@
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="89" t="str">
-        <x:v>Use this workbook to prove how the company generates revenue before building the Milestone 3 valuation model.</x:v>
+        <x:v>Complete all nine visible sheets, review Checks &amp; Submission, then upload this .xlsx for Stage 2.</x:v>
       </x:c>
       <x:c r="B2" s="89"/>
       <x:c r="C2" s="89"/>
@@ -892,7 +892,7 @@
         <x:v>Workbook version</x:v>
       </x:c>
       <x:c r="E6" s="84" t="str">
-        <x:v>1.0</x:v>
+        <x:v>1.5.0</x:v>
       </x:c>
       <x:c r="F6" s="91"/>
       <x:c r="G6" s="91"/>
@@ -908,7 +908,7 @@
         <x:v>Updated</x:v>
       </x:c>
       <x:c r="E7" s="84" t="str">
-        <x:v>2026-07-29</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
       <x:c r="F7" s="91"/>
       <x:c r="G7" s="91"/>
@@ -1913,7 +1913,7 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="9" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="21" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="31" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
@@ -2228,8 +2228,8 @@
       <x:c r="K19" s="92"/>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="82" t="str">
-        <x:v>Latest-year reported revenue change</x:v>
+      <x:c r="A20" s="94" t="str">
+        <x:v>Reported revenue change</x:v>
       </x:c>
       <x:c r="B20" s="111" t="str">
         <x:f>IF(OR('Revenue History'!G6="",'Revenue History'!H6=""),"",'Revenue History'!H6-'Revenue History'!G6)</x:f>
@@ -2249,8 +2249,8 @@
       <x:c r="K20" s="114"/>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="82" t="str">
-        <x:v>Total quantified driver effects</x:v>
+      <x:c r="A21" s="94" t="str">
+        <x:v>Quantified driver effects</x:v>
       </x:c>
       <x:c r="B21" s="111" t="n">
         <x:f>SUM(F6:F17)</x:f>
@@ -2271,8 +2271,8 @@
       <x:c r="K21" s="114"/>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="82" t="str">
-        <x:v>Unexplained / directional remainder</x:v>
+      <x:c r="A22" s="94" t="str">
+        <x:v>Directional remainder</x:v>
       </x:c>
       <x:c r="B22" s="111" t="str">
         <x:f>IF(B20="","",B20-B21)</x:f>
@@ -2292,7 +2292,7 @@
       <x:c r="K22" s="114"/>
     </x:row>
     <x:row r="23">
-      <x:c r="A23" s="82" t="str">
+      <x:c r="A23" s="94" t="str">
         <x:v>Bridge status</x:v>
       </x:c>
       <x:c r="B23" s="113" t="str">
@@ -2314,7 +2314,7 @@
       <x:c r="K23" s="114"/>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="82" t="str">
+      <x:c r="A24" s="94" t="str">
         <x:v>Management interpretation</x:v>
       </x:c>
       <x:c r="B24" s="83" t="str"/>

</xml_diff>